<commit_message>
modulo de envio masivo
</commit_message>
<xml_diff>
--- a/migracion/Clientes.xlsx
+++ b/migracion/Clientes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\DesarrolloWeb358\gestion-global\migracion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904D42C7-17F4-4727-AB3D-08ABF083A9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B376DF2C-4223-4883-9969-BA977CE758F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,10 +37,10 @@
     <t/>
   </si>
   <si>
-    <t>AGRUPACIÓN DE VIVIENDA BUENOS AIRES II SECTOR PRIMERA ETAPA - P.H.</t>
-  </si>
-  <si>
-    <t>agrupacionbuenosaires@gmail.com</t>
+    <t>CONJUNTO RESIDENCIAL ANTURIO I - P.H.</t>
+  </si>
+  <si>
+    <t>conjuntoanturio1@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -132,9 +132,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -511,18 +509,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:25" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2">
-        <v>800240183</v>
+        <v>900727994</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="2">
-        <v>800240183</v>
+        <v>900727994</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -548,7 +546,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="mailto:agrupacionbuenosaires@gmail.com" xr:uid="{66339381-21D3-4B8A-9BC3-980B48FBCF66}"/>
+    <hyperlink ref="C2" r:id="rId1" display="mailto:conjuntoanturio1@gmail.com" xr:uid="{203A4AEE-7C69-464D-B990-26DC51F7C66E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>